<commit_message>
Add word "afsløring" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -493,9 +493,77 @@
         <v>Lapses</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>404b4586-544a-4f23-b918-5b4822c01e86</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-12</v>
+      </c>
+      <c r="C2" t="str">
+        <v>afsløring</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F2" t="str">
+        <v>en</v>
+      </c>
+      <c r="G2" t="str">
+        <v>-en, -er, -erneBøjningsformerafsløringenafsløringerafsløringerne</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[-ˌsløˀɐ̯eŋ]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000721_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>1. opdagelse af et (uhæderligt) forhold som har været forsøgt skjultPå få måneder har tolderne i forbindelse med 20 afsløringer konfiskeret 428.000 cigaretter JyP1992Morgenavisen Jyllands-Posten (avis), 1992.2. undersøgelse og omtale af forhold der h</v>
+      </c>
+      <c r="K2" t="str">
+        <v>disclosure</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Efter Ingeniøren-afsløring: Novo Nordisk ramt af »uautoriseret adgang« til interne it-systemer</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Efter Ingeniøren-afsløring: Novo Nordisk ramt af »uautoriseret adgang« til interne it-systemer | Ingeniøren</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://ing.dk/artikel/efter-ingenioeren-afsloering-novo-nordisk-ramt-af-uautoriseret-adgang-til-interne-it-systemer</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://ing.dk/artikel/efter-ingenioeren-afsloering-novo-nordisk-ramt-af-uautoriseret-adgang-til-interne-it-systemer#:~:text=afsl%C3%B8ring</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -504,22 +572,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,8 +651,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "ramt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -561,9 +561,77 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>99c81e31-6d8a-4f91-b372-1bb3d35bed1c</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-06-12</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ramt</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>-t, -meBøjningsformerramtramme</v>
+      </c>
+      <c r="H3" t="str">
+        <v>[ˈʁɑmˀ]</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://static.ordnet.dk/mp3/11042/11042079_1.mp3</v>
+      </c>
+      <c r="J3" t="str">
+        <v xml:space="preserve">1. skarp, bitter eller stram; som minder om gæring eller forrådnelse om lugt eller smagOrd i nærhedenulækkerbeskharsksur2råddenkrasbitter2 Henter ... Henter ... Eksemplerram lugtEn ram og sødlig pislugt breder sig fra ham BeRasm89Bent Rasmussen: Den </v>
+      </c>
+      <c r="K3" t="str">
+        <v>hit</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Efter Ingeniøren-afsløring: Novo Nordisk ramt af »uautoriseret adgang« til interne it-systemer</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Efter Ingeniøren-afsløring: Novo Nordisk ramt af »uautoriseret adgang« til interne it-systemer | Ingeniøren</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://ing.dk/artikel/efter-ingenioeren-afsloering-novo-nordisk-ramt-af-uautoriseret-adgang-til-interne-it-systemer</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://ing.dk/artikel/efter-ingenioeren-afsloering-novo-nordisk-ramt-af-uautoriseret-adgang-til-interne-it-systemer#:~:text=ramt</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress for 2 cards in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -401,28 +401,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V3"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,19 +546,19 @@
         <v>ok</v>
       </c>
       <c r="R2" t="str">
-        <v/>
+        <v>2026-06-12</v>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="U2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="V2" t="str">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -614,19 +614,19 @@
         <v>ok</v>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>2026-06-12</v>
       </c>
       <c r="S3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="T3" t="str">
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="U3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="V3" t="str">
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phone: add 1 entry in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,30 +399,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,9 +629,77 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>289ac26a-cc77-4d82-a6b5-1937ed0aabc6</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-06-12</v>
+      </c>
+      <c r="C4" t="str">
+        <v>patientoplysninger</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>pending</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress for 1 card in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -620,7 +620,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="str">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="U3" t="str">
         <v>0</v>

</xml_diff>

<commit_message>
Add word "konstateret" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,30 +399,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -697,9 +697,77 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>14ef19a1-f118-4e23-878b-6eb6ddb8d7fa</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-06-12</v>
+      </c>
+      <c r="C5" t="str">
+        <v>konstateret</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>-r, -de, -tBøjningsformerkonstatererkonstateredekonstateret</v>
+      </c>
+      <c r="H5" t="str">
+        <v>[kʌnsdaˈteˀʌ]</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://static.ordnet.dk/mp3/11027/11027406_1.mp3</v>
+      </c>
+      <c r="J5" t="str">
+        <v>1. slå fast som en kendsgerning; påviseOrd i nærhedenvidne omtale sit eget/tydelige sprogfastslåfundereunderbyggebelægge med Henter ... Henter ... grammatikNOGEN konstaterer NOGET/at+SÆTNINGKun i ca. 500 tilfælde årligt vil dødens indtræden blive kon</v>
+      </c>
+      <c r="K5" t="str">
+        <v>ascertained</v>
+      </c>
+      <c r="L5" t="str">
+        <v>»Novo Nordisk A/S har for nylig konstateret en it-sikkerhedshændelse, der involverede uautoriseret adgang til et begrænset antal interne it-systemer. Hændelsen omfattede uautoriseret adgang til visse personoplysninger, der var lagret på de interne it-systemer.«</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Efter Ingeniøren-afsløring: Novo Nordisk ramt af »uautoriseret adgang« til interne it-systemer | Ingeniøren</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://ing.dk/artikel/efter-ingenioeren-afsloering-novo-nordisk-ramt-af-uautoriseret-adgang-til-interne-it-systemer</v>
+      </c>
+      <c r="O5" t="str">
+        <v>https://ing.dk/artikel/efter-ingenioeren-afsloering-novo-nordisk-ramt-af-uautoriseret-adgang-til-interne-it-systemer#:~:text=konstateret</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Enrich 1 pending entry in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -401,28 +401,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V5"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -661,7 +661,7 @@
         <v/>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>Patient information</v>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -679,7 +679,7 @@
         <v/>
       </c>
       <c r="Q4" t="str">
-        <v>pending</v>
+        <v>partial</v>
       </c>
       <c r="R4" t="str">
         <v/>

</xml_diff>

<commit_message>
Add word "overvismand" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,30 +399,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -765,9 +765,77 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>41bf7a9c-2396-4cb2-a539-018da128066a</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C6" t="str">
+        <v>overvismand</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F6" t="str">
+        <v>en</v>
+      </c>
+      <c r="G6" t="str">
+        <v>-en, ..mænd, ..mændeneBøjningsformerovervismanden..mænd..mændene</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>https://static.ordnet.dk/mp3/50007/50007015_1.mp3</v>
+      </c>
+      <c r="J6" t="str">
+        <v xml:space="preserve">formand for de økonomiske vismænd, dvs. formandskabet i De Økonomiske Råd, hvis opgave er at rådgive regering og folketing i samfundsøkonomiske anliggenderOrd i nærhedennationaløkonomsamfundsøkonomøkonommonetarist Henter ... Henter ... Overvismanden </v>
+      </c>
+      <c r="K6" t="str">
+        <v>Overseer</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Hvornår kan vi mærke AI-revolutionen på pengepungen? Vi har spurgt Danmarks økonomiske overvismand</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O6" t="str">
+        <v>https://ing.dk/#:~:text=overvismand</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forbud" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -833,9 +833,77 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>6edb0700-f46c-4fa5-a380-7745917e85d3</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C7" t="str">
+        <v>forbud</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F7" t="str">
+        <v>et</v>
+      </c>
+      <c r="G7" t="str">
+        <v>-det (eller uofficiel form: -et), -, -dene (eller uofficiel form: -ene) Se bøjning i skemaBøjningsformerforbuddet (eller uofficiel form: forbudet)forbudforbuddene (eller uofficiel form: forbudene)Bemæ</v>
+      </c>
+      <c r="H7" t="str">
+        <v>[ˈfɒːˌbuð]</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014300_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v>bestemmelse om at noget ikke må finde sted eller ikke må forekommeAntonym tilladelseSe også påbudOrd i nærhedenlovbestemmelseulovlighed Henter ... Henter ... grammatiknedlægge forbud mod at../NOGET få forbud mod at../NOGETEksemplergenerelt forbudtota</v>
+      </c>
+      <c r="K7" t="str">
+        <v>prohibition</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Bruger du amerikansk tech? Trumps seneste AI-forbud er et wakup-call</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Forurenede vandløb var under restaurering for millioner - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O7" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=forbud</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress for 5 cards in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -546,13 +546,13 @@
         <v>ok</v>
       </c>
       <c r="R2" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-17</v>
       </c>
       <c r="S2" t="str">
         <v>0</v>
       </c>
       <c r="T2" t="str">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="U2" t="str">
         <v>0</v>
@@ -614,16 +614,16 @@
         <v>ok</v>
       </c>
       <c r="R3" t="str">
-        <v>2026-06-17</v>
+        <v>2026-06-18</v>
       </c>
       <c r="S3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" t="str">
         <v>1.3</v>
       </c>
       <c r="U3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V3" t="str">
         <v>0</v>
@@ -682,16 +682,16 @@
         <v>partial</v>
       </c>
       <c r="R4" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-18</v>
       </c>
       <c r="S4" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4" t="str">
         <v>2.3</v>
       </c>
       <c r="U4" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V4" t="str">
         <v>0</v>
@@ -818,19 +818,19 @@
         <v>ok</v>
       </c>
       <c r="R6" t="str">
-        <v/>
+        <v>2026-06-17</v>
       </c>
       <c r="S6" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="T6" t="str">
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="U6" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="V6" t="str">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -886,19 +886,19 @@
         <v>ok</v>
       </c>
       <c r="R7" t="str">
-        <v/>
+        <v>2026-06-18</v>
       </c>
       <c r="S7" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="T7" t="str">
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="U7" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="V7" t="str">
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add word "burde" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -122,10 +122,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -157,10 +157,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -570,9 +570,77 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>1cb69bc1-7dde-4225-b376-ffb92920b0af</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C3" t="str">
+        <v>burde</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>bør, -, -tBøjningsformerbørburdeburdet</v>
+      </c>
+      <c r="H3" t="str">
+        <v>[ˈboɐ̯də]</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://static.ordnet.dk/mp3/11006/11006756_1.mp3</v>
+      </c>
+      <c r="J3" t="str">
+        <v xml:space="preserve">1. være påkrævet fordi det er tilrådeligt, rimeligt eller moralsk rigtigtSe også skullemåtteOrd i nærhedenmåtte2være nødt tilhave meget at se tilvære nødsaget tilse sig nødsaget tilføle sig nødsaget til Henter ... Henter ... grammatikNOGEN/NOGET bør </v>
+      </c>
+      <c r="K3" t="str">
+        <v>should</v>
+      </c>
+      <c r="L3" t="str">
+        <v>»Når unge cykler i hverdagen, får de bevægelse ind som en naturlig del af dagen uden at skulle sætte ekstra tid af til motion. Det er så sundt at cykle, at man burde udskrive det på recept.«</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=burde</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add word "udskrive" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -122,10 +122,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -157,10 +157,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -638,9 +638,77 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>8317ce8e-18d6-47d1-bce0-08a349c15f36</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C4" t="str">
+        <v>udskrive</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>-r, udskrev, udskrevetBøjningsformerudskriverudskrevudskrevet præteritum participium brugt som foranstillet adjektiv: udskreven eller udskrevet, udskrevet, udskrevne Se bøjning i skemaBøjningsformerud</v>
+      </c>
+      <c r="H4" t="str">
+        <v>[ˈuðˌsgʁiˀvə]</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004113_1.mp3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>1. udmelde og sende hjem fra en institution el.lign., især et hospital, efter endt behandlingSe også indlæggeOrd i nærhedenkurere Henter ... Henter ... grammatikNOGEN udskriver NOGENEksemplerblive udskrevetmange patienter bliver udskrevet allerede to</v>
+      </c>
+      <c r="K4" t="str">
+        <v>print</v>
+      </c>
+      <c r="L4" t="str">
+        <v>»Når unge cykler i hverdagen, får de bevægelse ind som en naturlig del af dagen uden at skulle sætte ekstra tid af til motion. Det er så sundt at cykle, at man burde udskrive det på recept.«</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="O4" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=udskrive</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add phrase "udskrive det på recept" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Words" sheetId="2" r:id="rId2"/>
+    <sheet name="Phrases" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -122,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -157,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -410,28 +411,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V4"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -711,4 +712,133 @@
     <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>DateAdded</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Phrase</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Gloss</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Translation</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Snippet</v>
+      </c>
+      <c r="G1" t="str">
+        <v>SourceTitle</v>
+      </c>
+      <c r="H1" t="str">
+        <v>SourceURL</v>
+      </c>
+      <c r="I1" t="str">
+        <v>DeepLink</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Note</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Due</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Interval</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Ease</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Reps</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Lapses</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>d6d91258-6089-4611-8c73-51946d14e419</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C2" t="str">
+        <v>udskrive det på recept</v>
+      </c>
+      <c r="D2" t="str">
+        <v>udskrive=print · det=the · på=on · recept=prescription</v>
+      </c>
+      <c r="E2" t="str">
+        <v>print it on prescription</v>
+      </c>
+      <c r="F2" t="str">
+        <v>»Når unge cykler i hverdagen, får de bevægelse ind som en naturlig del af dagen uden at skulle sætte ekstra tid af til motion. Det er så sundt at cykle, at man burde udskrive det på recept.«</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=udskrive%20det%20p%C3%A5%20recept</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add phrase "I forvejen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -716,7 +716,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -836,9 +836,59 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>27f40ec3-0006-43bd-bbc3-7629e481d89f</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C3" t="str">
+        <v>I forvejen</v>
+      </c>
+      <c r="D3" t="str">
+        <v>I=In · forvejen=in advance</v>
+      </c>
+      <c r="E3" t="str">
+        <v>In advance</v>
+      </c>
+      <c r="F3" t="str">
+        <v>I forvejen bliver cyklen fravalgt af stadig flere unge. Tal fra Syddansk Universitet viser, at andelen, der cykler til arbejde eller uddannelse mindst tre gange om ugen, er faldet. Tilbagegangen er særlig markant blandt unge: Blandt de 15-19-årige er cyklingen faldet med 16 pct.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="H3" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=I%20forvejen</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add word "fravalgt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -409,30 +409,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -707,9 +707,77 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>49fec14f-e37f-4cc3-b92d-14b281bdbc93</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C5" t="str">
+        <v>fravalgt</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>-r, fravalgte, fravalgtBøjningsformerfravælgerfravalgtefravalgt</v>
+      </c>
+      <c r="H5" t="str">
+        <v>[-ˌvεlˀjə]</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://static.ordnet.dk/mp3/11015/11015768_1.mp3</v>
+      </c>
+      <c r="J5" t="str">
+        <v>undlade at vælge noget bestemt, evt. sådan at man derved automatisk vælger noget andetSynonymer vælge frasjældent bortvælgeSe også tilvælgeOrd i nærhedenvælgevælge frabortvælgestemme nogen hjem Henter ... Henter ... grammatikNOGEN fravælger NOGETvi [</v>
+      </c>
+      <c r="K5" t="str">
+        <v>deselected</v>
+      </c>
+      <c r="L5" t="str">
+        <v>I forvejen bliver cyklen fravalgt af stadig flere unge. Tal fra Syddansk Universitet viser, at andelen, der cykler til arbejde eller uddannelse mindst tre gange om ugen, er faldet. Tilbagegangen er særlig markant blandt unge: Blandt de 15-19-årige er cyklingen faldet med 16 pct.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="O5" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=fravalgt</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -718,22 +786,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P3"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "forvejen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -775,9 +775,77 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>e4c4b72f-79f9-44ad-9f7d-e769da8c31f0</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C6" t="str">
+        <v>forvejen</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F6" t="str">
+        <v>en</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>[ˈfɒːˌvɑjˀən]</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://static.ordnet.dk/mp3/11015/11015503_1.mp3</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>in advance</v>
+      </c>
+      <c r="L6" t="str">
+        <v>I forvejen bliver cyklen fravalgt af stadig flere unge. Tal fra Syddansk Universitet viser, at andelen, der cykler til arbejde eller uddannelse mindst tre gange om ugen, er faldet. Tilbagegangen er særlig markant blandt unge: Blandt de 15-19-årige er cyklingen faldet med 16 pct.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="O6" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=forvejen</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "andelen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -843,9 +843,77 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>7881a1dd-2b75-43d1-8410-768a4f600067</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C7" t="str">
+        <v>andelen</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F7" t="str">
+        <v>en</v>
+      </c>
+      <c r="G7" t="str">
+        <v>-en, -e, -eneBøjningsformerandelenandeleandelene</v>
+      </c>
+      <c r="H7" t="str">
+        <v>[ˈanˌdeˀl]</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001671_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v xml:space="preserve">1. del, part eller udsnit af en bestemt mængde eller genstandOrd i nærhedenafdelingblok1grundenhedregiondelmængdehalvdel Henter ... Henter ... grammatikandel af NOGET få/have andel i NOGET andel på MÆNGDEEn dansk undersøgelse har vist, at andelen af </v>
+      </c>
+      <c r="K7" t="str">
+        <v>The share</v>
+      </c>
+      <c r="L7" t="str">
+        <v>I forvejen bliver cyklen fravalgt af stadig flere unge. Tal fra Syddansk Universitet viser, at andelen, der cykler til arbejde eller uddannelse mindst tre gange om ugen, er faldet. Tilbagegangen er særlig markant blandt unge: Blandt de 15-19-årige er cyklingen faldet med 16 pct.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="O7" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=andelen</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Tilbagegangen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -911,9 +911,77 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>282e62cf-c01c-46a8-896a-92c518032e29</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Tilbagegangen</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F8" t="str">
+        <v>en</v>
+      </c>
+      <c r="G8" t="str">
+        <v>-en, -e, -eneBøjningsformertilbagegangentilbagegangetilbagegangene</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>https://static.ordnet.dk/mp3/12001/12001025_1.mp3</v>
+      </c>
+      <c r="J8" t="str">
+        <v>1. fald i antal eller størrelseSynonym nedgangAntonym fremgangOrd i nærhedenaftagningregressionindskrumpningkrympningsvækkelseafsvækkelse Henter ... Henter ... grammatiktilbagegang i NOGET især i singularisEksemplervoldsom/kraftig tilbagegangvære i t</v>
+      </c>
+      <c r="K8" t="str">
+        <v>The decline</v>
+      </c>
+      <c r="L8" t="str">
+        <v>I forvejen bliver cyklen fravalgt af stadig flere unge. Tal fra Syddansk Universitet viser, at andelen, der cykler til arbejde eller uddannelse mindst tre gange om ugen, er faldet. Tilbagegangen er særlig markant blandt unge: Blandt de 15-19-årige er cyklingen faldet med 16 pct.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="N8" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="O8" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=Tilbagegangen</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "blandt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -979,9 +979,77 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>d3d68873-5ed4-47a6-a873-ce24d48d4af4</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="C9" t="str">
+        <v>blandt</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v>præposition</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>[bland]</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://static.ordnet.dk/mp3/11005/11005048_1.mp3</v>
+      </c>
+      <c r="J9" t="str">
+        <v>1. på eller til et sted inde midt i; omgivet afSynonymer mellemiblandtOrd i nærhedeniblandt2 Henter ... Henter ... Eksemplerblandt publikumblandt tilskuerneCharmen skrues der først op for, når han er blandt venner og familie BerlT1991Berlingske Tiden</v>
+      </c>
+      <c r="K9" t="str">
+        <v>among</v>
+      </c>
+      <c r="L9" t="str">
+        <v>I forvejen bliver cyklen fravalgt af stadig flere unge. Tal fra Syddansk Universitet viser, at andelen, der cykler til arbejde eller uddannelse mindst tre gange om ugen, er faldet. Tilbagegangen er særlig markant blandt unge: Blandt de 15-19-årige er cyklingen faldet med 16 pct.</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Cykelboss advarer: Gratis busbillet til unge er en tikkende bombe | Ingeniøren</v>
+      </c>
+      <c r="N9" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe</v>
+      </c>
+      <c r="O9" t="str">
+        <v>https://ing.dk/artikel/cykelboss-advarer-gratis-busbillet-til-unge-er-en-tikkende-bombe#:~:text=blandt</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "årige" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Nyheder.xlsx
+++ b/12-06-2026-vokab/Nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ